<commit_message>
📊 BIST Screener | 09.04.2026 16:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-09.xlsx
+++ b/data/bist_screener_2026-04-09.xlsx
@@ -25658,21 +25658,21 @@
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B580" s="3" t="n">
-        <v>36.1</v>
+        <v>68.2</v>
       </c>
       <c r="C580" s="4" t="n">
-        <v>-0.009899999999999999</v>
+        <v>0.1</v>
       </c>
       <c r="D580" s="5" t="n">
-        <v>5700000</v>
+        <v>4160000</v>
       </c>
       <c r="E580" s="2" t="inlineStr"/>
       <c r="F580" s="3" t="n">
-        <v>49.11</v>
+        <v>60.26</v>
       </c>
       <c r="G580" s="2" t="inlineStr"/>
       <c r="H580" s="2" t="inlineStr"/>
@@ -25680,12 +25680,12 @@
       <c r="J580" s="2" t="inlineStr"/>
       <c r="K580" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L580" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M580" s="2" t="inlineStr"/>
@@ -25693,21 +25693,21 @@
     <row r="581">
       <c r="A581" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B581" s="7" t="n">
-        <v>23.06</v>
+        <v>6.22</v>
       </c>
       <c r="C581" s="8" t="n">
-        <v>-0.0162</v>
+        <v>0.006500000000000001</v>
       </c>
       <c r="D581" s="9" t="n">
-        <v>17230000</v>
+        <v>14530000</v>
       </c>
       <c r="E581" s="6" t="inlineStr"/>
       <c r="F581" s="7" t="n">
-        <v>52.29</v>
+        <v>85.28</v>
       </c>
       <c r="G581" s="6" t="inlineStr"/>
       <c r="H581" s="6" t="inlineStr"/>
@@ -25715,47 +25715,49 @@
       <c r="J581" s="6" t="inlineStr"/>
       <c r="K581" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L581" s="6" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L581" s="6" t="inlineStr"/>
       <c r="M581" s="6" t="inlineStr"/>
     </row>
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B582" s="3" t="n">
-        <v>2.85</v>
+        <v>158.4</v>
       </c>
       <c r="C582" s="4" t="n">
-        <v>-0.0104</v>
+        <v>0.0089</v>
       </c>
       <c r="D582" s="5" t="n">
-        <v>298200000</v>
-      </c>
-      <c r="E582" s="2" t="inlineStr"/>
+        <v>1120000</v>
+      </c>
+      <c r="E582" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F582" s="3" t="n">
-        <v>60.14</v>
+        <v>77.47</v>
       </c>
       <c r="G582" s="2" t="inlineStr"/>
       <c r="H582" s="2" t="inlineStr"/>
-      <c r="I582" s="2" t="inlineStr"/>
-      <c r="J582" s="2" t="inlineStr"/>
+      <c r="I582" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J582" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K582" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L582" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M582" s="2" t="inlineStr"/>
@@ -25763,59 +25765,61 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="C583" s="6" t="inlineStr"/>
-      <c r="D583" s="6" t="inlineStr"/>
-      <c r="E583" s="6" t="inlineStr"/>
-      <c r="F583" s="6" t="inlineStr"/>
+        <v>9.82</v>
+      </c>
+      <c r="C583" s="8" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="D583" s="7" t="n">
+        <v>257600</v>
+      </c>
+      <c r="E583" s="8" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F583" s="7" t="n">
+        <v>60.09</v>
+      </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
-      <c r="I583" s="6" t="inlineStr"/>
-      <c r="J583" s="6" t="inlineStr"/>
-      <c r="K583" s="6" t="inlineStr"/>
-      <c r="L583" s="6" t="inlineStr">
-        <is>
-          <t>BIST TÜM</t>
-        </is>
-      </c>
+      <c r="I583" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J583" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
+      <c r="K583" s="6" t="inlineStr">
+        <is>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L583" s="6" t="inlineStr"/>
       <c r="M583" s="6" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>68.2</v>
-      </c>
-      <c r="C584" s="4" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D584" s="5" t="n">
-        <v>4160000</v>
-      </c>
+        <v>23.2</v>
+      </c>
+      <c r="C584" s="2" t="inlineStr"/>
+      <c r="D584" s="2" t="inlineStr"/>
       <c r="E584" s="2" t="inlineStr"/>
-      <c r="F584" s="3" t="n">
-        <v>60.26</v>
-      </c>
+      <c r="F584" s="2" t="inlineStr"/>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
       <c r="I584" s="2" t="inlineStr"/>
       <c r="J584" s="2" t="inlineStr"/>
-      <c r="K584" s="2" t="inlineStr">
-        <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
+      <c r="K584" s="2" t="inlineStr"/>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TÜM</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25823,23 +25827,23 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>3.6</v>
+        <v>28.24</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>0.0405</v>
-      </c>
-      <c r="D585" s="7" t="n">
-        <v>64400000.00000001</v>
+        <v>0.0262</v>
+      </c>
+      <c r="D585" s="9" t="n">
+        <v>10730000</v>
       </c>
       <c r="E585" s="8" t="n">
-        <v>0.8667</v>
+        <v>0.2667</v>
       </c>
       <c r="F585" s="7" t="n">
-        <v>62.56</v>
+        <v>56.48</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
@@ -25847,12 +25851,12 @@
       <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25860,40 +25864,34 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>3.63</v>
+        <v>41.48</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.1</v>
+        <v>0.0058</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>37490000</v>
-      </c>
-      <c r="E586" s="4" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>21980000</v>
+      </c>
+      <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>71.72</v>
+        <v>56.48</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
-      <c r="I586" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J586" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I586" s="2" t="inlineStr"/>
+      <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25901,21 +25899,21 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>41.48</v>
+        <v>23.06</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0058</v>
+        <v>-0.0162</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>21980000</v>
+        <v>17230000</v>
       </c>
       <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>56.48</v>
+        <v>52.29</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25923,12 +25921,12 @@
       <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25936,34 +25934,40 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>173.3</v>
+        <v>3.42</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0643</v>
+        <v>0.0395</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>15410000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>74180000</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>73.42</v>
+        <v>69.36</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="I588" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J588" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25971,28 +25975,38 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>81.83</v>
+        <v>3.6</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0112</v>
-      </c>
-      <c r="D589" s="9" t="n">
-        <v>12700000</v>
-      </c>
-      <c r="E589" s="6" t="inlineStr"/>
+        <v>0.0405</v>
+      </c>
+      <c r="D589" s="7" t="n">
+        <v>64400000.00000001</v>
+      </c>
+      <c r="E589" s="8" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F589" s="7" t="n">
-        <v>42.88</v>
+        <v>62.56</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
       <c r="I589" s="6" t="inlineStr"/>
       <c r="J589" s="6" t="inlineStr"/>
-      <c r="K589" s="6" t="inlineStr"/>
-      <c r="L589" s="6" t="inlineStr"/>
+      <c r="K589" s="6" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
@@ -26037,97 +26051,93 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>9.82</v>
+        <v>173.3</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.096</v>
-      </c>
-      <c r="D591" s="7" t="n">
-        <v>257600</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>-0.0643</v>
+      </c>
+      <c r="D591" s="9" t="n">
+        <v>15410000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>60.09</v>
+        <v>73.42</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J591" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I591" s="6" t="inlineStr"/>
+      <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+        </is>
+      </c>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>81.5</v>
+        <v>36.1</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0578</v>
+        <v>-0.009899999999999999</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>22480</v>
-      </c>
-      <c r="E592" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>5700000</v>
+      </c>
+      <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>36.4</v>
+        <v>49.11</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J592" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I592" s="2" t="inlineStr"/>
+      <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>AKGRT</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>7.4</v>
+        <v>236.7</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.0109</v>
+        <v>-0.0138</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>11410000</v>
+        <v>8320</v>
       </c>
       <c r="E593" s="8" t="n">
-        <v>0.28</v>
+        <v>0.2578</v>
       </c>
       <c r="F593" s="7" t="n">
-        <v>47.66</v>
+        <v>37.36</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
@@ -26135,53 +26145,49 @@
       <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr"/>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>158.4</v>
+        <v>3.63</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.0089</v>
+        <v>0.1</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>1120000</v>
+        <v>37490000</v>
       </c>
       <c r="E594" s="4" t="n">
-        <v>0.1071</v>
+        <v>0.1672</v>
       </c>
       <c r="F594" s="3" t="n">
-        <v>77.47</v>
+        <v>71.72</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
       <c r="I594" s="4" t="n">
-        <v>-3.6635</v>
+        <v>-5.3262</v>
       </c>
       <c r="J594" s="4" t="n">
-        <v>-0.4897</v>
+        <v>-4.2562</v>
       </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26189,34 +26195,38 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>243</v>
+        <v>60.4</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.09859999999999999</v>
+        <v>-0.0139</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>10320000</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
+        <v>1010000</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F595" s="7" t="n">
-        <v>84.02</v>
+        <v>53.47</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="6" t="inlineStr"/>
+      <c r="J595" s="8" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26224,21 +26234,21 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>6.22</v>
+        <v>243</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.006500000000000001</v>
+        <v>0.09859999999999999</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>14530000</v>
+        <v>10320000</v>
       </c>
       <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>85.28</v>
+        <v>84.02</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26246,70 +26256,86 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>138.6</v>
+        <v>81.5</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.09939999999999999</v>
-      </c>
-      <c r="D597" s="6" t="inlineStr"/>
-      <c r="E597" s="6" t="inlineStr"/>
-      <c r="F597" s="6" t="inlineStr"/>
+        <v>-0.0578</v>
+      </c>
+      <c r="D597" s="9" t="n">
+        <v>22480</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F597" s="7" t="n">
+        <v>36.4</v>
+      </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="6" t="inlineStr"/>
-      <c r="K597" s="6" t="inlineStr"/>
+      <c r="I597" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J597" s="8" t="n">
+        <v>-4.155</v>
+      </c>
+      <c r="K597" s="6" t="inlineStr">
+        <is>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
       <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>AKGRT</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>5.93</v>
+        <v>7.4</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.09880000000000001</v>
+        <v>0.0109</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>150100000</v>
+        <v>11410000</v>
       </c>
       <c r="E598" s="4" t="n">
-        <v>0.2478</v>
+        <v>0.28</v>
       </c>
       <c r="F598" s="3" t="n">
-        <v>14.14</v>
+        <v>47.66</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
-      <c r="I598" s="4" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
+      <c r="I598" s="2" t="inlineStr"/>
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26317,23 +26343,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>236.7</v>
+        <v>13.58</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0138</v>
+        <v>-0.0181</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>8320</v>
-      </c>
-      <c r="E599" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>64940000</v>
+      </c>
+      <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>37.36</v>
+        <v>53.49</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26344,27 +26368,31 @@
           <t>İşlenebilen endüstriler</t>
         </is>
       </c>
-      <c r="L599" s="6" t="inlineStr"/>
+      <c r="L599" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>17.01</v>
+        <v>2.85</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.08449999999999999</v>
+        <v>-0.0104</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>131870000</v>
+        <v>298200000</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>55.39</v>
+        <v>60.14</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26377,7 +26405,7 @@
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26385,110 +26413,84 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>17.39</v>
+        <v>138.6</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0142</v>
-      </c>
-      <c r="D601" s="9" t="n">
-        <v>12780000</v>
-      </c>
-      <c r="E601" s="8" t="n">
-        <v>0.9246</v>
-      </c>
-      <c r="F601" s="7" t="n">
-        <v>48.59</v>
-      </c>
-      <c r="G601" s="7" t="n">
-        <v>164.37</v>
-      </c>
+        <v>-0.09939999999999999</v>
+      </c>
+      <c r="D601" s="6" t="inlineStr"/>
+      <c r="E601" s="6" t="inlineStr"/>
+      <c r="F601" s="6" t="inlineStr"/>
+      <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="8" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J601" s="8" t="n">
-        <v>-10.3171</v>
-      </c>
-      <c r="K601" s="6" t="inlineStr">
-        <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
-        </is>
-      </c>
+      <c r="I601" s="6" t="inlineStr"/>
+      <c r="J601" s="6" t="inlineStr"/>
+      <c r="K601" s="6" t="inlineStr"/>
+      <c r="L601" s="6" t="inlineStr"/>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>3.42</v>
+        <v>81.83</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0395</v>
+        <v>-0.0112</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>74180000</v>
-      </c>
-      <c r="E602" s="4" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>12700000</v>
+      </c>
+      <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>69.36</v>
+        <v>42.88</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J602" s="4" t="n">
-        <v>-0.8093</v>
-      </c>
-      <c r="K602" s="2" t="inlineStr">
-        <is>
-          <t>Dağıtım servisleri</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+      <c r="I602" s="2" t="inlineStr"/>
+      <c r="J602" s="2" t="inlineStr"/>
+      <c r="K602" s="2" t="inlineStr"/>
+      <c r="L602" s="2" t="inlineStr"/>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>33.24</v>
+        <v>17.39</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0154</v>
+        <v>-0.0142</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>5230000</v>
-      </c>
-      <c r="E603" s="6" t="inlineStr"/>
+        <v>12780000</v>
+      </c>
+      <c r="E603" s="8" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F603" s="7" t="n">
-        <v>54.32</v>
-      </c>
-      <c r="G603" s="6" t="inlineStr"/>
+        <v>48.59</v>
+      </c>
+      <c r="G603" s="7" t="n">
+        <v>164.37</v>
+      </c>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="6" t="inlineStr"/>
-      <c r="J603" s="6" t="inlineStr"/>
+      <c r="I603" s="8" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J603" s="8" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
           <t>Üretici imalatı</t>
@@ -26496,7 +26498,7 @@
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26504,38 +26506,38 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>60.4</v>
+        <v>5.93</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0139</v>
+        <v>-0.09880000000000001</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>1010000</v>
+        <v>150100000</v>
       </c>
       <c r="E604" s="4" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.2478</v>
       </c>
       <c r="F604" s="3" t="n">
-        <v>53.47</v>
+        <v>14.14</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="2" t="inlineStr"/>
-      <c r="J604" s="4" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="I604" s="4" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
+      <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26543,23 +26545,21 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>28.24</v>
+        <v>33.24</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0262</v>
+        <v>-0.0154</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>10730000</v>
-      </c>
-      <c r="E605" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>5230000</v>
+      </c>
+      <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>56.48</v>
+        <v>54.32</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26567,12 +26567,12 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26615,21 +26615,21 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>13.58</v>
+        <v>17.01</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0181</v>
+        <v>-0.08449999999999999</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>64940000</v>
+        <v>131870000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>53.49</v>
+        <v>55.39</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26637,12 +26637,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26669,7 +26669,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>09.04.2026 15:30</t>
+          <t>09.04.2026 16:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 09.04.2026 18:41 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-09.xlsx
+++ b/data/bist_screener_2026-04-09.xlsx
@@ -25658,21 +25658,21 @@
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B580" s="3" t="n">
-        <v>68.2</v>
+        <v>173.3</v>
       </c>
       <c r="C580" s="4" t="n">
-        <v>0.1</v>
+        <v>-0.0643</v>
       </c>
       <c r="D580" s="5" t="n">
-        <v>4160000</v>
+        <v>15410000</v>
       </c>
       <c r="E580" s="2" t="inlineStr"/>
       <c r="F580" s="3" t="n">
-        <v>60.26</v>
+        <v>73.42</v>
       </c>
       <c r="G580" s="2" t="inlineStr"/>
       <c r="H580" s="2" t="inlineStr"/>
@@ -25685,7 +25685,7 @@
       </c>
       <c r="L580" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M580" s="2" t="inlineStr"/>
@@ -25693,21 +25693,21 @@
     <row r="581">
       <c r="A581" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B581" s="7" t="n">
-        <v>6.22</v>
+        <v>41.48</v>
       </c>
       <c r="C581" s="8" t="n">
-        <v>0.006500000000000001</v>
+        <v>0.0058</v>
       </c>
       <c r="D581" s="9" t="n">
-        <v>14530000</v>
+        <v>21980000</v>
       </c>
       <c r="E581" s="6" t="inlineStr"/>
       <c r="F581" s="7" t="n">
-        <v>85.28</v>
+        <v>56.48</v>
       </c>
       <c r="G581" s="6" t="inlineStr"/>
       <c r="H581" s="6" t="inlineStr"/>
@@ -25715,49 +25715,47 @@
       <c r="J581" s="6" t="inlineStr"/>
       <c r="K581" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L581" s="6" t="inlineStr"/>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L581" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+        </is>
+      </c>
       <c r="M581" s="6" t="inlineStr"/>
     </row>
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B582" s="3" t="n">
-        <v>158.4</v>
+        <v>13.58</v>
       </c>
       <c r="C582" s="4" t="n">
-        <v>0.0089</v>
+        <v>-0.0181</v>
       </c>
       <c r="D582" s="5" t="n">
-        <v>1120000</v>
-      </c>
-      <c r="E582" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>64940000</v>
+      </c>
+      <c r="E582" s="2" t="inlineStr"/>
       <c r="F582" s="3" t="n">
-        <v>77.47</v>
+        <v>53.49</v>
       </c>
       <c r="G582" s="2" t="inlineStr"/>
       <c r="H582" s="2" t="inlineStr"/>
-      <c r="I582" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J582" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I582" s="2" t="inlineStr"/>
+      <c r="J582" s="2" t="inlineStr"/>
       <c r="K582" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L582" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M582" s="2" t="inlineStr"/>
@@ -25765,98 +25763,106 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>9.82</v>
+        <v>158.4</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>0.096</v>
-      </c>
-      <c r="D583" s="7" t="n">
-        <v>257600</v>
+        <v>0.0089</v>
+      </c>
+      <c r="D583" s="9" t="n">
+        <v>1120000</v>
       </c>
       <c r="E583" s="8" t="n">
-        <v>0.95</v>
+        <v>0.1071</v>
       </c>
       <c r="F583" s="7" t="n">
-        <v>60.09</v>
+        <v>77.47</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
       <c r="I583" s="8" t="n">
-        <v>-23.6291</v>
+        <v>-3.6635</v>
       </c>
       <c r="J583" s="8" t="n">
-        <v>-0.4678</v>
+        <v>-0.4897</v>
       </c>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L583" s="6" t="inlineStr"/>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L583" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+        </is>
+      </c>
       <c r="M583" s="6" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="C584" s="2" t="inlineStr"/>
-      <c r="D584" s="2" t="inlineStr"/>
+        <v>81.83</v>
+      </c>
+      <c r="C584" s="4" t="n">
+        <v>-0.0112</v>
+      </c>
+      <c r="D584" s="5" t="n">
+        <v>12700000</v>
+      </c>
       <c r="E584" s="2" t="inlineStr"/>
-      <c r="F584" s="2" t="inlineStr"/>
+      <c r="F584" s="3" t="n">
+        <v>42.88</v>
+      </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
       <c r="I584" s="2" t="inlineStr"/>
       <c r="J584" s="2" t="inlineStr"/>
       <c r="K584" s="2" t="inlineStr"/>
-      <c r="L584" s="2" t="inlineStr">
-        <is>
-          <t>BIST TÜM</t>
-        </is>
-      </c>
+      <c r="L584" s="2" t="inlineStr"/>
       <c r="M584" s="2" t="inlineStr"/>
     </row>
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>FENER</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>28.24</v>
+        <v>2.74</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>0.0262</v>
+        <v>-0.0352</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>10730000</v>
+        <v>94030000</v>
       </c>
       <c r="E585" s="8" t="n">
-        <v>0.2667</v>
+        <v>0.6898000000000001</v>
       </c>
       <c r="F585" s="7" t="n">
-        <v>56.48</v>
+        <v>46.32</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
       <c r="I585" s="6" t="inlineStr"/>
-      <c r="J585" s="6" t="inlineStr"/>
+      <c r="J585" s="8" t="n">
+        <v>-2.0083</v>
+      </c>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25864,21 +25870,21 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>41.48</v>
+        <v>2.85</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.0058</v>
+        <v>-0.0104</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>21980000</v>
+        <v>298200000</v>
       </c>
       <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>56.48</v>
+        <v>60.14</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
@@ -25886,12 +25892,12 @@
       <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25899,34 +25905,40 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>23.06</v>
+        <v>3.42</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.0162</v>
+        <v>0.0395</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>17230000</v>
-      </c>
-      <c r="E587" s="6" t="inlineStr"/>
+        <v>74180000</v>
+      </c>
+      <c r="E587" s="8" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F587" s="7" t="n">
-        <v>52.29</v>
+        <v>69.36</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="6" t="inlineStr"/>
-      <c r="J587" s="6" t="inlineStr"/>
+      <c r="I587" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J587" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25934,64 +25946,60 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>3.42</v>
+        <v>9.82</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0395</v>
-      </c>
-      <c r="D588" s="5" t="n">
-        <v>74180000</v>
+        <v>0.096</v>
+      </c>
+      <c r="D588" s="3" t="n">
+        <v>257600</v>
       </c>
       <c r="E588" s="4" t="n">
-        <v>0.7119</v>
+        <v>0.95</v>
       </c>
       <c r="F588" s="3" t="n">
-        <v>69.36</v>
+        <v>60.09</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="4" t="n">
-        <v>-191.6342</v>
+        <v>-23.6291</v>
       </c>
       <c r="J588" s="4" t="n">
-        <v>-0.8093</v>
+        <v>-0.4678</v>
       </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L588" s="2" t="inlineStr"/>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>3.6</v>
+        <v>236.7</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0405</v>
-      </c>
-      <c r="D589" s="7" t="n">
-        <v>64400000.00000001</v>
+        <v>-0.0138</v>
+      </c>
+      <c r="D589" s="9" t="n">
+        <v>8320</v>
       </c>
       <c r="E589" s="8" t="n">
-        <v>0.8667</v>
+        <v>0.2578</v>
       </c>
       <c r="F589" s="7" t="n">
-        <v>62.56</v>
+        <v>37.36</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -25999,73 +26007,55 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr"/>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>FENER</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>2.74</v>
+        <v>138.6</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0352</v>
-      </c>
-      <c r="D590" s="5" t="n">
-        <v>94030000</v>
-      </c>
-      <c r="E590" s="4" t="n">
-        <v>0.6898000000000001</v>
-      </c>
-      <c r="F590" s="3" t="n">
-        <v>46.32</v>
-      </c>
+        <v>-0.09939999999999999</v>
+      </c>
+      <c r="D590" s="2" t="inlineStr"/>
+      <c r="E590" s="2" t="inlineStr"/>
+      <c r="F590" s="2" t="inlineStr"/>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="2" t="inlineStr"/>
-      <c r="J590" s="4" t="n">
-        <v>-2.0083</v>
-      </c>
-      <c r="K590" s="2" t="inlineStr">
-        <is>
-          <t>Tüketici hizmetleri</t>
-        </is>
-      </c>
-      <c r="L590" s="2" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
-        </is>
-      </c>
+      <c r="J590" s="2" t="inlineStr"/>
+      <c r="K590" s="2" t="inlineStr"/>
+      <c r="L590" s="2" t="inlineStr"/>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>173.3</v>
+        <v>28.24</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0643</v>
+        <v>0.0262</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>15410000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>10730000</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>73.42</v>
+        <v>56.48</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26073,12 +26063,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26086,108 +26076,112 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>36.1</v>
+        <v>81.5</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.009899999999999999</v>
+        <v>-0.0578</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>5700000</v>
-      </c>
-      <c r="E592" s="2" t="inlineStr"/>
+        <v>22480</v>
+      </c>
+      <c r="E592" s="4" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F592" s="3" t="n">
-        <v>49.11</v>
+        <v>36.4</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="2" t="inlineStr"/>
-      <c r="J592" s="2" t="inlineStr"/>
+      <c r="I592" s="4" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J592" s="4" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr"/>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>236.7</v>
+        <v>3.63</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0138</v>
+        <v>0.1</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>8320</v>
+        <v>37490000</v>
       </c>
       <c r="E593" s="8" t="n">
-        <v>0.2578</v>
+        <v>0.1672</v>
       </c>
       <c r="F593" s="7" t="n">
-        <v>37.36</v>
+        <v>71.72</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="6" t="inlineStr"/>
-      <c r="J593" s="6" t="inlineStr"/>
+      <c r="I593" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J593" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>3.63</v>
+        <v>23.06</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.1</v>
+        <v>-0.0162</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>37490000</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>17230000</v>
+      </c>
+      <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>71.72</v>
+        <v>52.29</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J594" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I594" s="2" t="inlineStr"/>
+      <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26195,38 +26189,36 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>60.4</v>
+        <v>3.6</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0139</v>
-      </c>
-      <c r="D595" s="9" t="n">
-        <v>1010000</v>
+        <v>0.0405</v>
+      </c>
+      <c r="D595" s="7" t="n">
+        <v>64400000.00000001</v>
       </c>
       <c r="E595" s="8" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.8667</v>
       </c>
       <c r="F595" s="7" t="n">
-        <v>53.47</v>
+        <v>62.56</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="8" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26269,60 +26261,60 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>81.5</v>
+        <v>5.93</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0578</v>
+        <v>-0.09880000000000001</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>22480</v>
+        <v>150100000</v>
       </c>
       <c r="E597" s="8" t="n">
-        <v>0.58</v>
+        <v>0.2478</v>
       </c>
       <c r="F597" s="7" t="n">
-        <v>36.4</v>
+        <v>14.14</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
       <c r="I597" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J597" s="8" t="n">
-        <v>-4.155</v>
-      </c>
+        <v>-0.0005999999999999999</v>
+      </c>
+      <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr"/>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
+        </is>
+      </c>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>AKGRT</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>7.4</v>
+        <v>33.24</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.0109</v>
+        <v>-0.0154</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>11410000</v>
-      </c>
-      <c r="E598" s="4" t="n">
-        <v>0.28</v>
-      </c>
+        <v>5230000</v>
+      </c>
+      <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>47.66</v>
+        <v>54.32</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26330,12 +26322,12 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26343,34 +26335,38 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>13.58</v>
+        <v>60.4</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0181</v>
+        <v>-0.0139</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>64940000</v>
-      </c>
-      <c r="E599" s="6" t="inlineStr"/>
+        <v>1010000</v>
+      </c>
+      <c r="E599" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F599" s="7" t="n">
-        <v>53.49</v>
+        <v>53.47</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
       <c r="I599" s="6" t="inlineStr"/>
-      <c r="J599" s="6" t="inlineStr"/>
+      <c r="J599" s="8" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26378,21 +26374,21 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>SVGYO</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>2.85</v>
+        <v>16.89</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.0104</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>298200000</v>
+        <v>114920000</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>60.14</v>
+        <v>86.78</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26405,7 +26401,7 @@
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26413,131 +26409,145 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>138.6</v>
+        <v>36.1</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.09939999999999999</v>
-      </c>
-      <c r="D601" s="6" t="inlineStr"/>
+        <v>-0.009899999999999999</v>
+      </c>
+      <c r="D601" s="9" t="n">
+        <v>5700000</v>
+      </c>
       <c r="E601" s="6" t="inlineStr"/>
-      <c r="F601" s="6" t="inlineStr"/>
+      <c r="F601" s="7" t="n">
+        <v>49.11</v>
+      </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="6" t="inlineStr"/>
       <c r="J601" s="6" t="inlineStr"/>
-      <c r="K601" s="6" t="inlineStr"/>
-      <c r="L601" s="6" t="inlineStr"/>
+      <c r="K601" s="6" t="inlineStr">
+        <is>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>81.83</v>
+        <v>17.39</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0112</v>
+        <v>-0.0142</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>12700000</v>
-      </c>
-      <c r="E602" s="2" t="inlineStr"/>
+        <v>12780000</v>
+      </c>
+      <c r="E602" s="4" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F602" s="3" t="n">
-        <v>42.88</v>
-      </c>
-      <c r="G602" s="2" t="inlineStr"/>
+        <v>48.59</v>
+      </c>
+      <c r="G602" s="3" t="n">
+        <v>164.37</v>
+      </c>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="2" t="inlineStr"/>
-      <c r="J602" s="2" t="inlineStr"/>
-      <c r="K602" s="2" t="inlineStr"/>
-      <c r="L602" s="2" t="inlineStr"/>
+      <c r="I602" s="4" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J602" s="4" t="n">
+        <v>-10.3171</v>
+      </c>
+      <c r="K602" s="2" t="inlineStr">
+        <is>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>17.39</v>
+        <v>6.22</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0142</v>
+        <v>0.006500000000000001</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>12780000</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>14530000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>48.59</v>
-      </c>
-      <c r="G603" s="7" t="n">
-        <v>164.37</v>
-      </c>
+        <v>85.28</v>
+      </c>
+      <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr"/>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>AKGRT</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>5.93</v>
+        <v>7.4</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.09880000000000001</v>
+        <v>0.0109</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>150100000</v>
+        <v>11410000</v>
       </c>
       <c r="E604" s="4" t="n">
-        <v>0.2478</v>
+        <v>0.28</v>
       </c>
       <c r="F604" s="3" t="n">
-        <v>14.14</v>
+        <v>47.66</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="4" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
+      <c r="I604" s="2" t="inlineStr"/>
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26545,21 +26555,21 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>33.24</v>
+        <v>68.2</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.0154</v>
+        <v>0.1</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>5230000</v>
+        <v>4160000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>54.32</v>
+        <v>60.26</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26567,12 +26577,12 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26580,34 +26590,24 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>SVGYO</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>16.89</v>
-      </c>
-      <c r="C606" s="4" t="n">
-        <v>0.09960000000000001</v>
-      </c>
-      <c r="D606" s="5" t="n">
-        <v>114920000</v>
-      </c>
+        <v>23.2</v>
+      </c>
+      <c r="C606" s="2" t="inlineStr"/>
+      <c r="D606" s="2" t="inlineStr"/>
       <c r="E606" s="2" t="inlineStr"/>
-      <c r="F606" s="3" t="n">
-        <v>86.78</v>
-      </c>
+      <c r="F606" s="2" t="inlineStr"/>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
       <c r="I606" s="2" t="inlineStr"/>
       <c r="J606" s="2" t="inlineStr"/>
-      <c r="K606" s="2" t="inlineStr">
-        <is>
-          <t>Finans</t>
-        </is>
-      </c>
+      <c r="K606" s="2" t="inlineStr"/>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
+          <t>BIST TÜM</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26669,7 +26669,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>09.04.2026 16:30</t>
+          <t>09.04.2026 18:41</t>
         </is>
       </c>
     </row>

</xml_diff>